<commit_message>
feat(supplementary): ensure Supplementary Files 2 and 3 are 100% verbatim identical to runtime prompt strings in annotation_prompts.py
</commit_message>
<xml_diff>
--- a/publication/manuscripts/Supplementary_File_2_FAERS_Annotation_Guidance.xlsx
+++ b/publication/manuscripts/Supplementary_File_2_FAERS_Annotation_Guidance.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="11">
+  <fonts count="10">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,12 +75,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="001B365D"/>
-      <sz val="9.5"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <i val="1"/>
-      <sz val="9"/>
+      <sz val="10"/>
     </font>
   </fonts>
   <fills count="6">
@@ -141,7 +136,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" indent="1"/>
@@ -189,17 +184,20 @@
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -566,7 +564,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G12"/>
+  <dimension ref="B2:G13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -588,11 +586,11 @@
     <row r="3" ht="24" customHeight="1">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Complete 17-Category Schema, Operational Annotation Rules, Trigger Phrases, and Clinical Exemplars</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="22" customHeight="1">
+          <t>Exact Verbatim Annotation Schema and Operational Rules Injected into LLM Prompts</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="24" customHeight="1">
       <c r="B5" s="3" t="inlineStr">
         <is>
           <t>Supplementary File:</t>
@@ -608,7 +606,7 @@
       <c r="F5" s="5" t="n"/>
       <c r="G5" s="5" t="n"/>
     </row>
-    <row r="6" ht="22" customHeight="1">
+    <row r="6" ht="24" customHeight="1">
       <c r="B6" s="3" t="inlineStr">
         <is>
           <t>Document Title:</t>
@@ -624,7 +622,7 @@
       <c r="F6" s="5" t="n"/>
       <c r="G6" s="5" t="n"/>
     </row>
-    <row r="7" ht="22" customHeight="1">
+    <row r="7" ht="24" customHeight="1">
       <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Associated Manuscript:</t>
@@ -640,7 +638,7 @@
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
     </row>
-    <row r="8" ht="22" customHeight="1">
+    <row r="8" ht="24" customHeight="1">
       <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Target Corpus:</t>
@@ -648,7 +646,7 @@
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>FDA Adverse Event Reporting System (FAERS) Case Series Benchmark (N = 829 Narratives)</t>
+          <t>FDA Adverse Event Reporting System (FAERS) Benchmark (N = 829 Narratives)</t>
         </is>
       </c>
       <c r="D8" s="5" t="n"/>
@@ -656,15 +654,15 @@
       <c r="F8" s="5" t="n"/>
       <c r="G8" s="5" t="n"/>
     </row>
-    <row r="9" ht="22" customHeight="1">
+    <row r="9" ht="24" customHeight="1">
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Total Concept Categories:</t>
+          <t>Total Categories:</t>
         </is>
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>17 Primary Clinical Concept Categories</t>
+          <t>17 Primary Clinical Concept Categories (Exact Verbatim Prompt Schema)</t>
         </is>
       </c>
       <c r="D9" s="5" t="n"/>
@@ -672,15 +670,15 @@
       <c r="F9" s="5" t="n"/>
       <c r="G9" s="5" t="n"/>
     </row>
-    <row r="10" ht="22" customHeight="1">
+    <row r="10" ht="24" customHeight="1">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Category Breakdown:</t>
+          <t>In-Text XML Tags:</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>sDrug, cDrug, oDrug, Dose, IND, Treatment, AE, mAE, Dx, Lab, Status, R/O, CoD, MHx, FHx, Age, Sex</t>
+          <t>&lt;SDRUG&gt;, &lt;CDRUG&gt;, &lt;ODRUG&gt;, &lt;DOSE&gt;, &lt;IND&gt;, &lt;TREATMENT&gt;, &lt;AE&gt;, &lt;MAE&gt;, &lt;DX&gt;, &lt;LAB&gt;, &lt;STATUS&gt;, &lt;RO&gt;, &lt;COD&gt;, &lt;MHX&gt;, &lt;FHX&gt;, &lt;AGE&gt;, &lt;SEX&gt;</t>
         </is>
       </c>
       <c r="D10" s="5" t="n"/>
@@ -688,17 +686,15 @@
       <c r="F10" s="5" t="n"/>
       <c r="G10" s="5" t="n"/>
     </row>
-    <row r="11" ht="22" customHeight="1">
+    <row r="11" ht="24" customHeight="1">
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Evaluation Metric Tiers:</t>
+          <t>Structured JSON Keys:</t>
         </is>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Tier 1: Strict Exact-Match NER (CoNLL exact boundary + exact label)
-Tier 2: Adapted ADE-Eval (Clinical partial overlap + cross-class weighted credit)
-Tier 3: Relaxed Boundary (Token-level category agreement)</t>
+          <t>sdrug, cdrug, odrug, dose, ind, treatment, ae, mae, dx, lab, status, ro, cod, mhx, fhx, age, sex</t>
         </is>
       </c>
       <c r="D11" s="5" t="n"/>
@@ -706,15 +702,15 @@
       <c r="F11" s="5" t="n"/>
       <c r="G11" s="5" t="n"/>
     </row>
-    <row r="12" ht="22" customHeight="1">
+    <row r="12" ht="24" customHeight="1">
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Version &amp; Date:</t>
+          <t>Evaluation Protocol:</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Revision 1 (August 2026)</t>
+          <t>4-Fold Leave-One-Drug-Event-Pair-Out on BioBERT vs. Zero-Shot/1-Shot Instruction-Tuned LLMs (LLaMA 4 &amp; Claude 4.6 Sonnet)</t>
         </is>
       </c>
       <c r="D12" s="5" t="n"/>
@@ -722,8 +718,24 @@
       <c r="F12" s="5" t="n"/>
       <c r="G12" s="5" t="n"/>
     </row>
+    <row r="13" ht="24" customHeight="1">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Version &amp; Date:</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Revision 1 (August 2026)</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n"/>
+      <c r="E13" s="5" t="n"/>
+      <c r="F13" s="5" t="n"/>
+      <c r="G13" s="5" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="10">
+  <mergeCells count="11">
     <mergeCell ref="B3:G3"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="C7:G7"/>
@@ -732,6 +744,7 @@
     <mergeCell ref="C10:G10"/>
     <mergeCell ref="C11:G11"/>
     <mergeCell ref="C5:G5"/>
+    <mergeCell ref="C13:G13"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="C9:G9"/>
   </mergeCells>
@@ -745,24 +758,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:I21"/>
+  <dimension ref="B2:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
-    <col width="42" customWidth="1" min="6" max="6"/>
-    <col width="32" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
-    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="48" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>FAERS 17 Clinical Concept Category Annotation Schema</t>
+          <t>FAERS 17 Clinical Concept Category Annotation Schema (Verbatim LLM Prompt)</t>
         </is>
       </c>
     </row>
@@ -784,27 +795,17 @@
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Clinical Definition</t>
+          <t>Definition (Verbatim Prompt Text)</t>
         </is>
       </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
-          <t>Annotation Rule &amp; Scope</t>
+          <t>Annotation Rule (Verbatim Prompt Text)</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Trigger Words / Contextual Clues</t>
-        </is>
-      </c>
-      <c r="H4" s="8" t="inlineStr">
-        <is>
-          <t>Prototypical Clinical Examples</t>
-        </is>
-      </c>
-      <c r="I4" s="8" t="inlineStr">
-        <is>
-          <t>Classification Caveats &amp; Boundaries</t>
+          <t>Trigger Words / Contextual Clues (Verbatim Prompt Text)</t>
         </is>
       </c>
     </row>
@@ -826,28 +827,17 @@
       </c>
       <c r="E5" s="12" t="inlineStr">
         <is>
-          <t>A drug or biological product believed to have caused, contributed to, or been associated with the reported adverse event. Often discontinued, modified, interrupted, or rechallenged. May have explicit causal language linking it to the AE.</t>
+          <t>A drug or biological product believed to have caused, contributed to, or been associated with the adverse event. Often discontinued, changed, or adjusted after the AE. May have explicit causal language linking it to the AE.</t>
         </is>
       </c>
       <c r="F5" s="12" t="inlineStr">
         <is>
-          <t>Annotate a drug as sDrug when it is explicitly or strongly linked to the AE through causal, temporal, or attribution language. Clinical dechallenge (stopping/reducing drug) or rechallenge actions supporting causality also qualify.</t>
+          <t>Annotate a drug as **sDrug** when it is explicitly or strongly linked to the AE through causal, temporal, or attribution language. A clinical action taken because of the suspected relationship, such as discontinuation, dose reduction, dose increase, interruption, or rechallenge, can also support classification as sDrug.</t>
         </is>
       </c>
       <c r="G5" s="12" t="inlineStr">
         <is>
-          <t>suspected, suspect, implicated, caused, linked to, attributed to, associated with, following administration of, after starting, induced by, resolved after stopping, dechallenge, rechallenge</t>
-        </is>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>• '...patient experienced severe rash after starting azacitidine [sDrug]'
-• '...hypoglycemia suspected to be caused by tramadol [sDrug]'</t>
-        </is>
-      </c>
-      <c r="I5" s="12" t="inlineStr">
-        <is>
-          <t>Do not annotate concomitant chronic medications as sDrug unless explicitly implicated in causing the current AE.</t>
+          <t>suspected, suspect, implicated, caused, linked to, attributed to, associated with, related to, following administration of, after starting, after receiving, induced by, resolved after stopping, improved after discontinuation, symptoms worsened after increasing dose, dechallenge, rechallenge</t>
         </is>
       </c>
     </row>
@@ -869,28 +859,17 @@
       </c>
       <c r="E6" s="16" t="inlineStr">
         <is>
-          <t>Drugs that were concurrently administered with other drugs (e.g., suspect drugs), as part of the patient's ongoing or routine regimen. May include chronic medications, maintenance therapy, or background treatments.</t>
+          <t>Drugs that were concurrently administered with other drugs (e.g., suspect drugs), as part of the patient's ongoing or routine regimen. May include chronic medications, maintenance therapy, or background treatments. Some may have a potential or implicit causal relationship with the AE, as per applicant report.</t>
         </is>
       </c>
       <c r="F6" s="16" t="inlineStr">
         <is>
-          <t>Annotate a drug as cDrug when described as taken concurrently with the suspect drug or as part of ongoing regimen, without sufficient evidence to classify as suspect drug or rescue treatment.</t>
+          <t>Annotate a drug as **cDrug** when it is described as being taken concurrently with the suspect drug or as part of the patient's ongoing medication regimen, without sufficient evidence to classify it as the suspect drug or as treatment for the reported event.</t>
         </is>
       </c>
       <c r="G6" s="16" t="inlineStr">
         <is>
-          <t>concomitant, concomitant medication, background therapy, chronic therapy, maintenance therapy, maintained on, patient's usual medications, home medications, taken concurrently</t>
-        </is>
-      </c>
-      <c r="H6" s="16" t="inlineStr">
-        <is>
-          <t>• 'Concomitant medications included lisinopril [cDrug] and atorvastatin [cDrug]'
-• '...maintained on background metformin [cDrug]'</t>
-        </is>
-      </c>
-      <c r="I6" s="16" t="inlineStr">
-        <is>
-          <t>If a drug was initiated specifically to treat an AE, annotate as Treatment, not cDrug.</t>
+          <t>concomitant, concomitant medication, concomitant drug, background therapy, chronic therapy, maintenance therapy, maintained on, patient's usual medications, current medications, home medications, taken concurrently, other medications included, medication regimen</t>
         </is>
       </c>
     </row>
@@ -912,28 +891,17 @@
       </c>
       <c r="E7" s="12" t="inlineStr">
         <is>
-          <t>Drugs mentioned but not clearly linked to the current adverse event, concomitant therapy, or an explicit treatment purpose. Includes illicit substances, prior historical drug use, or drug class references without a specified current clinical role.</t>
+          <t>Drugs mentioned but not clearly linked to the current adverse event, concomitant drugs or therapy, or an explicit treatment purpose. Illicit substances should also be included when mentioned. Typically includes historical drug use or drug references without a specified current clinical role.</t>
         </is>
       </c>
       <c r="F7" s="12" t="inlineStr">
         <is>
-          <t>Annotate a drug or substance as oDrug when mentioned but cannot be reliably classified as sDrug, cDrug, or Treatment. Include historical drug exposure, general drug class references, and recreational/illicit substances.</t>
+          <t>Annotate a drug or substance as **oDrug** when it is mentioned but cannot be reliably classified as sDrug, cDrug, or Treatment. Include historical drug exposure, general drug references, investigational drugs without a defined role in the current event, and illicit/non-medical substances.</t>
         </is>
       </c>
       <c r="G7" s="12" t="inlineStr">
         <is>
-          <t>illicit substances, recreational drug, substance use, past medications, previous medication, drug history, prior drug use, drug class, general drug reference, investigational drug</t>
-        </is>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>• 'The patient had a history of cocaine [oDrug] use'
-• '...previously received multiple NSAIDs [oDrug] in childhood'</t>
-        </is>
-      </c>
-      <c r="I7" s="12" t="inlineStr">
-        <is>
-          <t>Do not use oDrug if the drug's role as suspect, concomitant, or treatment is explicitly stated.</t>
+          <t>illicit substances, recreational drug, substance use, past medications, previous medication, drug history, prior drug use, drug class, general drug reference, drug under investigation, investigational drug, historical use</t>
         </is>
       </c>
     </row>
@@ -955,28 +923,17 @@
       </c>
       <c r="E8" s="16" t="inlineStr">
         <is>
-          <t>Explicitly stated dosage information, strength, quantity, frequency, administration regimen, or stated dose adjustment associated with a drug product.</t>
+          <t>Explicitly stated dosage information associated with a drug.</t>
         </is>
       </c>
       <c r="F8" s="16" t="inlineStr">
         <is>
-          <t>Annotate the dosage information itself, not the drug name. Capture strength, unit, route descriptor, frequency, and dose modification descriptors when expressed together.</t>
+          <t>Annotate explicit dosage quantity, strength, frequency, regimen, or stated dose adjustment. Annotate the dosage information itself, not the drug name.</t>
         </is>
       </c>
       <c r="G8" s="16" t="inlineStr">
         <is>
-          <t>mg, mcg, g, mL, units, dose, dosage, once daily, twice daily, BID, TID, weekly, increased to, decreased to, reduced, titrated</t>
-        </is>
-      </c>
-      <c r="H8" s="16" t="inlineStr">
-        <is>
-          <t>• '...started on azacitidine 75 mg/m2 daily [Dose] for 7 days'
-• '...tramadol 50 mg every 6 hours [Dose]'</t>
-        </is>
-      </c>
-      <c r="I8" s="16" t="inlineStr">
-        <is>
-          <t>Do not include the drug name inside the Dose tag; keep drug name under sDrug/cDrug/Treatment.</t>
+          <t>mg, mcg, g, mL, units, dose, dosage, once daily, twice daily, BID, TID, weekly, increased, decreased, adjusted, reduced, titrated</t>
         </is>
       </c>
     </row>
@@ -998,28 +955,17 @@
       </c>
       <c r="E9" s="12" t="inlineStr">
         <is>
-          <t>The disease, condition, symptom, or intended medical purpose for which a drug, treatment, or procedure was prescribed, administered, or indicated.</t>
+          <t>The reason or intended medical purpose for which a drug, treatment, or procedure is used.</t>
         </is>
       </c>
       <c r="F9" s="12" t="inlineStr">
         <is>
-          <t>Annotate the condition, symptom, disease, or stated reason for which a drug or treatment was given. Include explicitly stated unknown or unspecified indications when clearly identified.</t>
+          <t>Annotate the condition, symptom, disease, or stated reason for which a drug, treatment, or procedure was given or intended. Include explicitly stated unknown or unspecified indications when clearly identified as the indication.</t>
         </is>
       </c>
       <c r="G9" s="12" t="inlineStr">
         <is>
-          <t>used for, given for, prescribed for, indicated for, to treat, for treatment of, for the management of, for prevention of, indication, reason for use</t>
-        </is>
-      </c>
-      <c r="H9" s="12" t="inlineStr">
-        <is>
-          <t>• 'Baricitinib was prescribed for rheumatoid arthritis [IND]'
-• '...erenumab indicated for migraine prophylaxis [IND]'</t>
-        </is>
-      </c>
-      <c r="I9" s="12" t="inlineStr">
-        <is>
-          <t>IND is the reason for medication; do not confuse with AE (the unwanted outcome) or Treatment (the therapy).</t>
+          <t>used for, given for, prescribed for, indicated for, to treat, for treatment of, for the management of, for prevention of, indication, reason for use, unknown indication</t>
         </is>
       </c>
     </row>
@@ -1031,7 +977,7 @@
       </c>
       <c r="C10" s="14" t="inlineStr">
         <is>
-          <t>Drug Used for Treatment</t>
+          <t>Drug used for treatment</t>
         </is>
       </c>
       <c r="D10" s="15" t="inlineStr">
@@ -1041,28 +987,17 @@
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>Drug products or medications explicitly described as treatments administered therapeutically to manage a disease, adverse event, complication, or symptom.</t>
+          <t>Drug products or drug administration explicitly described as treatments addressing disease, adverse events, complications, or symptoms.</t>
         </is>
       </c>
       <c r="F10" s="16" t="inlineStr">
         <is>
-          <t>Annotate a drug as Treatment only when explicitly administered or used therapeutically to manage a condition or rescue from an AE. Do not classify a drug as Treatment merely because it appears in a general medication list.</t>
+          <t>Annotate a drug as **Treatment** only when it is explicitly administered or used therapeutically to manage a disease, AE, complication, or symptom. Do not classify a drug as Treatment merely because it appears in a medication list.</t>
         </is>
       </c>
       <c r="G10" s="16" t="inlineStr">
         <is>
-          <t>treated with, treatment with, therapy with, was given, administered for, managed with, received, started on, prescribed to treat, rescue medication, supportive therapy</t>
-        </is>
-      </c>
-      <c r="H10" s="16" t="inlineStr">
-        <is>
-          <t>• 'The patient was treated with intravenous methylprednisolone [Treatment] for acute hypersensitivity'
-• '...received dextrose [Treatment] for severe hypoglycemia'</t>
-        </is>
-      </c>
-      <c r="I10" s="16" t="inlineStr">
-        <is>
-          <t>Pre-existing background medications belong to cDrug; only drugs given therapeutically to manage conditions/events are Treatment.</t>
+          <t>treated with, treatment with, therapy with, was given, administered for, managed with, received, started on, prescribed to treat, supportive treatment, rescue medication</t>
         </is>
       </c>
     </row>
@@ -1084,28 +1019,17 @@
       </c>
       <c r="E11" s="12" t="inlineStr">
         <is>
-          <t>Any untoward medical occurrence, negative health outcome, condition, sign, or symptom that represents a reported adverse event, regardless of proven causality.</t>
+          <t>Any negative health outcome, condition, sign, or symptom that could represent an adverse event, regardless of proven relation to a drug.</t>
         </is>
       </c>
       <c r="F11" s="12" t="inlineStr">
         <is>
-          <t>Annotate clinically relevant negative health outcomes, diagnosed conditions, signs, or patient-reported symptoms representing an adverse event. Proven drug causality is not required.</t>
+          <t>Annotate clinically relevant negative health outcomes, diagnosed conditions, signs, or patient-reported symptoms representing an adverse event. Do not require proven drug causality.</t>
         </is>
       </c>
       <c r="G11" s="12" t="inlineStr">
         <is>
-          <t>adverse event, developed, experienced, complained of, reports, diagnosed with, presented with, onset of, occurred, after starting, suffered, toxicity</t>
-        </is>
-      </c>
-      <c r="H11" s="12" t="inlineStr">
-        <is>
-          <t>• '...patient developed QT prolongation [AE] and syncope [AE]'
-• '...experienced an acute anaphylactic reaction [AE]'</t>
-        </is>
-      </c>
-      <c r="I11" s="12" t="inlineStr">
-        <is>
-          <t>Pre-existing conditions described as medical history belong to MHx, not AE.</t>
+          <t>adverse event, developed, experienced, complained of, reports, diagnosed with, presented with, onset of, occurred, after starting, unwell, discomfort</t>
         </is>
       </c>
     </row>
@@ -1117,7 +1041,7 @@
       </c>
       <c r="C12" s="14" t="inlineStr">
         <is>
-          <t>AE Manifestations / Sequelae</t>
+          <t>AE Manifestations/Sequelae</t>
         </is>
       </c>
       <c r="D12" s="15" t="inlineStr">
@@ -1127,28 +1051,17 @@
       </c>
       <c r="E12" s="16" t="inlineStr">
         <is>
-          <t>Immediate signs or symptoms occurring as explicit clinical manifestations of an identified AE, or secondary consequences, complications, and persistent sequelae resulting from an AE.</t>
+          <t>Manifestations are immediate signs or symptoms occurring as part of an identified AE. Sequelae are consequences, complications, or persistent secondary effects resulting from an AE.</t>
         </is>
       </c>
       <c r="F12" s="16" t="inlineStr">
         <is>
-          <t>Annotate a sign, symptom, clinical finding, or complication as mAE only when the narrative explicitly establishes it as a manifestation, complication, consequence, or sequela of another identified AE.</t>
+          <t>Annotate a sign, symptom, clinical finding, consequence, or complication as **mAE** only when the narrative explicitly establishes it as a manifestation, consequence, complication, or sequela of another identified AE. Do not infer this relationship solely from medical knowledge.</t>
         </is>
       </c>
       <c r="G12" s="16" t="inlineStr">
         <is>
-          <t>manifested as, symptoms included, characterized by, accompanied by, resulted in, complicated by, complication of, led to, secondary to, sequela, persistent</t>
-        </is>
-      </c>
-      <c r="H12" s="16" t="inlineStr">
-        <is>
-          <t>• '...developed severe hypoglycemia [AE] manifested by diaphoresis [mAE] and tremors [mAE]'
-• '...suffered a stroke [AE] resulting in hemiparesis [mAE]'</t>
-        </is>
-      </c>
-      <c r="I12" s="16" t="inlineStr">
-        <is>
-          <t>Do not infer mAE solely from medical intuition; explicit narrative link (e.g. 'manifested by', 'resulting in') is required.</t>
+          <t>manifested as, symptoms included, characterized by, accompanied by, resulted in, complicated by, complication of, led to, secondary to, sequela, persistent, residual, long-term effects</t>
         </is>
       </c>
     </row>
@@ -1170,28 +1083,17 @@
       </c>
       <c r="E13" s="12" t="inlineStr">
         <is>
-          <t>The name of a diagnostic imaging, endoscopic, electrophysiologic, biopsy, or exploratory procedure performed to evaluate or confirm a medical condition.</t>
+          <t>The name of a diagnostic procedure performed to evaluate or confirm a medical condition or diagnosis.</t>
         </is>
       </c>
       <c r="F13" s="12" t="inlineStr">
         <is>
-          <t>Annotate the diagnostic procedure itself. Do not annotate its resulting diagnosis or interpretation as Dx. Laboratory blood/urine tests belong under Lab.</t>
+          <t>Annotate the diagnostic procedure itself. Do not annotate its resulting diagnosis or interpretation as Dx. Laboratory tests and laboratory findings belong under Lab.</t>
         </is>
       </c>
       <c r="G13" s="12" t="inlineStr">
         <is>
-          <t>CT, CT scan, MRI, ultrasound, X-ray, radiograph, biopsy, histopathology, colonoscopy, endoscopy, echocardiogram, ECG, EKG, PET scan, angiography</t>
-        </is>
-      </c>
-      <c r="H13" s="12" t="inlineStr">
-        <is>
-          <t>• 'An emergency ECG [Dx] revealed prolonged QTc interval'
-• '...underwent brain MRI [Dx] confirming acute ischemia'</t>
-        </is>
-      </c>
-      <c r="I13" s="12" t="inlineStr">
-        <is>
-          <t>ECG/MRI/Biopsy are Dx; quantitative test values (e.g., QTc 520 ms) belong to Lab; the diagnosis (stroke) belongs to AE/sDx.</t>
+          <t>CT, CT scan, MRI, ultrasound, X-ray, radiograph, biopsy, histopathology, colonoscopy, endoscopy, echocardiogram, ECG, EKG, PET scan</t>
         </is>
       </c>
     </row>
@@ -1213,29 +1115,17 @@
       </c>
       <c r="E14" s="16" t="inlineStr">
         <is>
-          <t>Laboratory tests, clinical measurements, or quantitative/qualitative findings indicating objective clinical measurements (blood, urine, vitals, biomarkers, BMI, height, weight).</t>
+          <t>Laboratory tests, measurements, or results indicating quantitative or qualitative clinical findings.</t>
         </is>
       </c>
       <c r="F14" s="16" t="inlineStr">
         <is>
-          <t>Annotate laboratory test names and explicitly reported laboratory measurements/results, including normal, abnormal, elevated, positive, or negative findings.</t>
+          <t>Annotate laboratory test names and explicitly reported laboratory measurements/results, including normal, abnormal, positive, or negative findings. Objective measurements such as height, weight, and BMI may also be included when reported as clinical measurements.</t>
         </is>
       </c>
       <c r="G14" s="16" t="inlineStr">
         <is>
-          <t>result, level, value, measurement, elevated, increased, decreased, high, low, abnormal, normal, positive, negative, hemoglobin, platelet count, WBC, ALT, AST, creatinine, glucose, QTc</t>
-        </is>
-      </c>
-      <c r="H14" s="16" t="inlineStr">
-        <is>
-          <t>• 'Serum glucose was 32 mg/dL [Lab]'
-• '...platelet count dropped to 18,000/mcL [Lab]'
-• '...ALT elevated at 450 U/L [Lab]'</t>
-        </is>
-      </c>
-      <c r="I14" s="16" t="inlineStr">
-        <is>
-          <t>Diagnostic imaging procedures (CT, MRI) belong to Dx; quantitative lab tests and numeric values belong to Lab.</t>
+          <t>result, level, value, measurement, elevated, increased, decreased, high, low, abnormal, normal, positive, negative, hemoglobin, platelet count, WBC, ALT, AST, bilirubin, creatinine, urinalysis, serum, height, weight, BMI</t>
         </is>
       </c>
     </row>
@@ -1247,7 +1137,7 @@
       </c>
       <c r="C15" s="10" t="inlineStr">
         <is>
-          <t>Patient Status / Outcome</t>
+          <t>Patient Status</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1257,28 +1147,17 @@
       </c>
       <c r="E15" s="12" t="inlineStr">
         <is>
-          <t>Statements describing progression, clinical course, disposition, or outcome of the patient's overall clinical condition or adverse event following intervention.</t>
+          <t>Statements describing progression or outcome of the patient's overall clinical condition or an adverse event after treatment or intervention.</t>
         </is>
       </c>
       <c r="F15" s="12" t="inlineStr">
         <is>
-          <t>Annotate clinical course, recovery, deterioration, stability, persistence, hospitalization, admission, or discharge. Status describes what happened to the patient/event over time.</t>
+          <t>Annotate the clinical course, progression, outcome, recovery, deterioration, stability, persistence, or resolution. Status describes what happened to the patient or event rather than naming the underlying event itself.</t>
         </is>
       </c>
       <c r="G15" s="12" t="inlineStr">
         <is>
-          <t>recovered, resolved, improved, worsened, deteriorated, stable, unchanged, persistent, ongoing, outcome, admitted, discharged, hospitalized, asymptomatic, in remission</t>
-        </is>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
-        <is>
-          <t>• 'Symptoms completely resolved [Status] within 48 hours'
-• '...the patient was admitted to the ICU [Status] in critical condition [Status]'</t>
-        </is>
-      </c>
-      <c r="I15" s="12" t="inlineStr">
-        <is>
-          <t>Do not label the underlying disease name as Status; annotate the recovery/outcome descriptor itself.</t>
+          <t>recovered, resolved, improved, worsened, deteriorated, stable, unchanged, persistent, ongoing, outcome, admitted, discharged, hospitalized, asymptomatic, returned to baseline</t>
         </is>
       </c>
     </row>
@@ -1300,28 +1179,17 @@
       </c>
       <c r="E16" s="16" t="inlineStr">
         <is>
-          <t>Conditions, diseases, or differential diagnoses explicitly considered by clinicians but ultimately ruled out, excluded, or determined unsupported by findings.</t>
+          <t>Conditions considered but ultimately ruled out as explanations for symptoms or adverse events.</t>
         </is>
       </c>
       <c r="F16" s="16" t="inlineStr">
         <is>
-          <t>Annotate the condition or diagnosis that is explicitly ruled out or excluded. Do not classify a condition as R/O merely because a test is negative unless explicitly stated as excluded.</t>
+          <t>Annotate the condition or diagnosis that is explicitly ruled out, excluded, or determined unsupported. Do not automatically classify a condition as R/O solely because a test is negative.</t>
         </is>
       </c>
       <c r="G16" s="16" t="inlineStr">
         <is>
-          <t>ruled out, rule out, R/O, excluded, no evidence of, was considered but excluded, unlikely, not consistent with, negative for</t>
-        </is>
-      </c>
-      <c r="H16" s="16" t="inlineStr">
-        <is>
-          <t>• 'Infectious etiology was ruled out [R/O: infectious etiology]'
-• '...CT showed no evidence of intracranial hemorrhage [R/O: intracranial hemorrhage]'</t>
-        </is>
-      </c>
-      <c r="I16" s="16" t="inlineStr">
-        <is>
-          <t>Annotate the excluded disease concept, not the trigger phrase 'ruled out'.</t>
+          <t>ruled out, rule out, R/O, excluded, no evidence of, was considered but excluded, unlikely, not consistent with</t>
         </is>
       </c>
     </row>
@@ -1343,28 +1211,17 @@
       </c>
       <c r="E17" s="12" t="inlineStr">
         <is>
-          <t>A specific disease, condition, event, or clinical mechanism explicitly identified as causing or contributing to the patient's death.</t>
+          <t>A specific disease, condition, event, or reason explicitly identified as causing or contributing to the patient's death.</t>
         </is>
       </c>
       <c r="F17" s="12" t="inlineStr">
         <is>
-          <t>Annotate the stated cause or contributing cause of death. Do not annotate the single word 'death' alone unless it represents the stated causal concept.</t>
+          <t>Annotate the stated cause or contributing cause of death. Do not annotate the word "death" alone unless it itself represents the stated causal concept.</t>
         </is>
       </c>
       <c r="G17" s="12" t="inlineStr">
         <is>
-          <t>cause of death, died from, died of, death due to, death secondary to, succumbed to, resulted in death, fatal outcome attributed to</t>
-        </is>
-      </c>
-      <c r="H17" s="12" t="inlineStr">
-        <is>
-          <t>• 'The patient died from refractory cardiogenic shock [CoD]'
-• '...autopsy revealed massive pulmonary embolism [CoD] as the cause of death'</t>
-        </is>
-      </c>
-      <c r="I17" s="12" t="inlineStr">
-        <is>
-          <t>The fact of death/mortality status belongs to Status ('died'); the specific etiologic disease causing death is CoD.</t>
+          <t>cause of death, died from, died of, death due to, death secondary to, succumbed to, resulted in death, contributing cause of death</t>
         </is>
       </c>
     </row>
@@ -1386,28 +1243,17 @@
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>Symptoms, conditions, diseases, or medical findings that pre-existed before the current adverse event and were not caused by the suspect medication.</t>
+          <t>Symptoms, conditions, diagnoses, or medical findings that pre-existed before the current adverse event and were not caused by it.</t>
         </is>
       </c>
       <c r="F18" s="16" t="inlineStr">
         <is>
-          <t>Annotate the pre-existing or historical clinical condition itself. Do not include contextual phrases such as 'history of' when the condition can be captured separately.</t>
+          <t>Annotate the pre-existing or historical clinical condition itself. Do not include contextual phrases such as "history of" when the actual condition can be separately captured.</t>
         </is>
       </c>
       <c r="G18" s="16" t="inlineStr">
         <is>
           <t>past medical history, medical history, PMH, history of, baseline, chronic, prior diagnosis, pre-existing, underlying condition, known condition, longstanding</t>
-        </is>
-      </c>
-      <c r="H18" s="16" t="inlineStr">
-        <is>
-          <t>• 'Past medical history was notable for type 2 diabetes [MHx] and hypertension [MHx]'
-• '...a known history of severe asthma [MHx]'</t>
-        </is>
-      </c>
-      <c r="I18" s="16" t="inlineStr">
-        <is>
-          <t>Acute events occurring after drug initiation belong to AE; baseline pre-existing diseases belong to MHx.</t>
         </is>
       </c>
     </row>
@@ -1429,7 +1275,7 @@
       </c>
       <c r="E19" s="12" t="inlineStr">
         <is>
-          <t>Medical conditions, genetic disorders, or clinically relevant findings explicitly attributed to the patient's family members or family pedigree.</t>
+          <t>Medical conditions or clinically relevant findings attributed to the patient's family members or family history.</t>
         </is>
       </c>
       <c r="F19" s="12" t="inlineStr">
@@ -1439,18 +1285,7 @@
       </c>
       <c r="G19" s="12" t="inlineStr">
         <is>
-          <t>family history, FHx, mother had, father had, sibling had, family pedigree, familial, inherited, hereditary, genetic predisposition</t>
-        </is>
-      </c>
-      <c r="H19" s="12" t="inlineStr">
-        <is>
-          <t>• 'Family history was significant for early myocardial infarction [FHx] in father'
-• '...maternal aunt had breast cancer [FHx]'</t>
-        </is>
-      </c>
-      <c r="I19" s="12" t="inlineStr">
-        <is>
-          <t>Only diseases in family members qualify as FHx; the patient's own history is MHx.</t>
+          <t>family history, FHx, mother had, father had, sibling had, familial, inherited, hereditary, genetic predisposition</t>
         </is>
       </c>
     </row>
@@ -1462,7 +1297,7 @@
       </c>
       <c r="C20" s="14" t="inlineStr">
         <is>
-          <t>Patient Age</t>
+          <t>Age</t>
         </is>
       </c>
       <c r="D20" s="15" t="inlineStr">
@@ -1472,28 +1307,17 @@
       </c>
       <c r="E20" s="16" t="inlineStr">
         <is>
-          <t>The age or age category of the patient during the described adverse event episode.</t>
+          <t>The age or age category of the patient during the described event.</t>
         </is>
       </c>
       <c r="F20" s="16" t="inlineStr">
         <is>
-          <t>Annotate explicit references to the patient's exact age, age in years/months/days, or age category (pediatric, elderly). Annotate only references clearly applying to the patient.</t>
+          <t>Annotate explicit references to the patient's exact or approximate age or age category. Annotate only references that clearly refer to the patient.</t>
         </is>
       </c>
       <c r="G20" s="16" t="inlineStr">
         <is>
-          <t>year-old, years old, aged, age, adult, elderly, adolescent, child, pediatric, infant, newborn, neonate, octogenarian</t>
-        </is>
-      </c>
-      <c r="H20" s="16" t="inlineStr">
-        <is>
-          <t>• 'A 64-year-old [Age] male presented with...'
-• '...in an elderly [Age] patient with renal failure'</t>
-        </is>
-      </c>
-      <c r="I20" s="16" t="inlineStr">
-        <is>
-          <t>Do not annotate age mentions of relatives or other non-patient individuals.</t>
+          <t>year-old, years old, aged, age, adult, elderly, adolescent, child, pediatric, infant, newborn, neonate</t>
         </is>
       </c>
     </row>
@@ -1505,7 +1329,7 @@
       </c>
       <c r="C21" s="10" t="inlineStr">
         <is>
-          <t>Patient Sex</t>
+          <t>Sex</t>
         </is>
       </c>
       <c r="D21" s="11" t="inlineStr">
@@ -1515,7 +1339,7 @@
       </c>
       <c r="E21" s="12" t="inlineStr">
         <is>
-          <t>The biological sex or gender designation of the patient as explicitly described in the clinical narrative.</t>
+          <t>The biological sex of the patient as explicitly described in the clinical narrative.</t>
         </is>
       </c>
       <c r="F21" s="12" t="inlineStr">
@@ -1525,24 +1349,13 @@
       </c>
       <c r="G21" s="12" t="inlineStr">
         <is>
-          <t>male, female, man, woman, boy, girl, gentleman, lady</t>
-        </is>
-      </c>
-      <c r="H21" s="12" t="inlineStr">
-        <is>
-          <t>• 'A 45-year-old female [Sex] was admitted...'
-• '...the gentleman [Sex] experienced severe dizziness'</t>
-        </is>
-      </c>
-      <c r="I21" s="12" t="inlineStr">
-        <is>
-          <t>Do not annotate gender words referring to clinicians, family members, or bystanders.</t>
+          <t>male, female, man, woman, boy, girl</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="B2:I2"/>
+    <mergeCell ref="B2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1554,213 +1367,258 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:D14"/>
+  <dimension ref="B2:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="2" ht="30" customHeight="1">
       <c r="B2" s="6" t="inlineStr">
         <is>
-          <t>FAERS General Annotation Principles &amp; Operational Guidelines</t>
+          <t>FAERS General Annotation Rules &amp; Operational Principles (Verbatim LLM Prompt)</t>
         </is>
       </c>
     </row>
     <row r="4" ht="26" customHeight="1">
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>Rule # &amp; Principle</t>
-        </is>
-      </c>
-      <c r="C4" s="8" t="inlineStr">
-        <is>
-          <t>Operational Annotation Rule &amp; Clinical Rationale</t>
-        </is>
-      </c>
-      <c r="D4" s="8" t="inlineStr">
-        <is>
-          <t>Illustrative Case Examples</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="55" customHeight="1">
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>1. Contextual Role over Keyword Matching</t>
-        </is>
-      </c>
-      <c r="C5" s="12" t="inlineStr">
-        <is>
-          <t>Trigger words and phrases serve as contextual clues only; they do not automatically dictate an entity category. The annotator must evaluate the semantic and clinical role of each word in its specific narrative sentence.</t>
-        </is>
-      </c>
-      <c r="D5" s="18" t="inlineStr">
-        <is>
-          <t>Example: 'Rash' is an AE when occurring after medication, an IND when stated as the reason for treatment, and an MHx when reported in baseline history.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="55" customHeight="1">
-      <c r="B6" s="19" t="inlineStr">
-        <is>
-          <t>2. Minimal Clinically Meaningful Span</t>
-        </is>
-      </c>
-      <c r="C6" s="16" t="inlineStr">
-        <is>
-          <t>Annotate the smallest complete clinically informative span. Exclude unnecessary surrounding articles, conjunctions, prepositions, and contextual verbs.</t>
-        </is>
-      </c>
-      <c r="D6" s="20" t="inlineStr">
-        <is>
-          <t>Correct: 'treated with &lt;TREATMENT&gt;prednisone&lt;/TREATMENT&gt;'
-Incorrect: '&lt;TREATMENT&gt;treated with prednisone&lt;/TREATMENT&gt;'</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="55" customHeight="1">
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>3. Verbatim Exact Offsets</t>
-        </is>
-      </c>
-      <c r="C7" s="12" t="inlineStr">
-        <is>
-          <t>Every annotated span must match the source text character-by-character without spelling normalization, punctuation alteration, case folding, or lemmatization.</t>
-        </is>
-      </c>
-      <c r="D7" s="18" t="inlineStr">
-        <is>
-          <t>Preserve exact narrative characters: 'azacitidine 75mg/m2' must not be expanded or corrected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="55" customHeight="1">
-      <c r="B8" s="19" t="inlineStr">
-        <is>
-          <t>4. Non-Overlapping &amp; Non-Nested Policy</t>
-        </is>
-      </c>
-      <c r="C8" s="16" t="inlineStr">
-        <is>
-          <t>No text span may be assigned multiple overlapping or nested entity tags. If a phrase contains multiple concepts, choose the most specific primary role or segment into adjacent distinct spans.</t>
-        </is>
-      </c>
-      <c r="D8" s="20" t="inlineStr">
-        <is>
-          <t>In 'atenolol 25 mg', segment as '&lt;CDRUG&gt;atenolol&lt;/CDRUG&gt; &lt;DOSE&gt;25 mg&lt;/DOSE&gt;' rather than one nested tag.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="55" customHeight="1">
-      <c r="B9" s="17" t="inlineStr">
-        <is>
-          <t>5. Drug Precedence Hierarchy</t>
-        </is>
-      </c>
-      <c r="C9" s="12" t="inlineStr">
-        <is>
-          <t>Every drug mention must be resolved into exactly one of four mutually exclusive roles: (a) sDrug if suspect/implicated, (b) Treatment if administered to treat a condition/AE, (c) cDrug if concurrent/background regimen, or (d) oDrug if role is unspecified or historical.</t>
-        </is>
-      </c>
-      <c r="D9" s="18" t="inlineStr">
-        <is>
-          <t>A drug given in emergency for anaphylaxis is Treatment; the cancer chemotherapy suspected of causing anaphylaxis is sDrug.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="55" customHeight="1">
-      <c r="B10" s="19" t="inlineStr">
-        <is>
-          <t>6. AE vs. mAE Causality Constraint</t>
-        </is>
-      </c>
-      <c r="C10" s="16" t="inlineStr">
-        <is>
-          <t>Classify as mAE only when the narrative explicitly articulates a direct manifestation, secondary complication, or sequela relationship to a parent AE (e.g., 'manifested by', 'complicated by').</t>
-        </is>
-      </c>
-      <c r="D10" s="20" t="inlineStr">
-        <is>
-          <t>Do not infer mAE based solely on pathophysiology without textual linkage.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="55" customHeight="1">
-      <c r="B11" s="17" t="inlineStr">
-        <is>
-          <t>7. Temporal Separation: AE vs. MHx</t>
-        </is>
-      </c>
-      <c r="C11" s="12" t="inlineStr">
-        <is>
-          <t>A condition described as baseline, chronic, longstanding, or pre-existing prior to suspect medication initiation must be classified as MHx, whereas acute onset conditions post-administration are AE.</t>
-        </is>
-      </c>
-      <c r="D11" s="18" t="inlineStr">
-        <is>
-          <t>Baseline 'chronic kidney disease' = MHx; acute post-dose 'renal failure' = AE.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="55" customHeight="1">
-      <c r="B12" s="19" t="inlineStr">
-        <is>
-          <t>8. Indication (IND) vs. Treatment Disambiguation</t>
-        </is>
-      </c>
-      <c r="C12" s="16" t="inlineStr">
-        <is>
-          <t>IND is the underlying pathology or clinical purpose motivating medication use, whereas Treatment is the therapeutic agent or intervention applied.</t>
-        </is>
-      </c>
-      <c r="D12" s="20" t="inlineStr">
-        <is>
-          <t>In 'prednisone for eczema', 'prednisone' is Treatment and 'eczema' is IND.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="55" customHeight="1">
-      <c r="B13" s="17" t="inlineStr">
-        <is>
-          <t>9. Diagnostic Procedure (Dx) vs. Laboratory Finding (Lab)</t>
-        </is>
-      </c>
-      <c r="C13" s="12" t="inlineStr">
-        <is>
-          <t>Dx refers to imaging, exploratory procedures, endoscopies, and biopsies. Lab refers to clinical measurements, serum/urine tests, vital signs, quantitative values, and laboratory interpretation.</t>
-        </is>
-      </c>
-      <c r="D13" s="18" t="inlineStr">
-        <is>
-          <t>ECG is Dx; QTc interval 510 ms is Lab.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="55" customHeight="1">
-      <c r="B14" s="19" t="inlineStr">
-        <is>
-          <t>10. Patient Status vs. Underlying Disease</t>
-        </is>
-      </c>
-      <c r="C14" s="16" t="inlineStr">
-        <is>
-          <t>Status captures recovery trajectory, clinical course, admission, and discharge disposition. Do not annotate the disease name itself as Status.</t>
-        </is>
-      </c>
-      <c r="D14" s="20" t="inlineStr">
-        <is>
-          <t>In 'the patient fully recovered from hepatitis', 'recovered' is Status; 'hepatitis' is AE.</t>
-        </is>
-      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>Rule Number &amp; Principle</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>Operational Annotation Instruction (Verbatim Prompt Text)</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="n"/>
+    </row>
+    <row r="5" ht="50" customHeight="1">
+      <c r="B5" s="18" t="inlineStr">
+        <is>
+          <t>1. Use narrative context, not keyword matching.</t>
+        </is>
+      </c>
+      <c r="C5" s="19" t="inlineStr">
+        <is>
+          <t>Trigger words and phrases are contextual clues only. A trigger word does not automatically determine an annotation.</t>
+        </is>
+      </c>
+      <c r="D5" s="5" t="n"/>
+    </row>
+    <row r="6" ht="50" customHeight="1">
+      <c r="B6" s="20" t="inlineStr">
+        <is>
+          <t>2. Annotate the clinical entity, not the contextual trigger phrase.</t>
+        </is>
+      </c>
+      <c r="C6" s="21" t="inlineStr">
+        <is>
+          <t>For example:
+- "treated with prednisone" -&gt; annotate "prednisone" as Treatment.
+- "history of hypertension" -&gt; annotate "hypertension" as MHx.
+- "CT showed..." -&gt; annotate "CT" as Dx when appropriate.</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n"/>
+    </row>
+    <row r="7" ht="50" customHeight="1">
+      <c r="B7" s="18" t="inlineStr">
+        <is>
+          <t>3. Use exact text spans.</t>
+        </is>
+      </c>
+      <c r="C7" s="19" t="inlineStr">
+        <is>
+          <t>Every annotated span must occur verbatim in the source narrative. Do not normalize spelling, capitalization, abbreviations, numbers, or units.</t>
+        </is>
+      </c>
+      <c r="D7" s="5" t="n"/>
+    </row>
+    <row r="8" ht="50" customHeight="1">
+      <c r="B8" s="20" t="inlineStr">
+        <is>
+          <t>4. Prefer the smallest complete clinically meaningful span.</t>
+        </is>
+      </c>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>Do not include unnecessary surrounding words, punctuation, conjunctions, or trigger phrases.</t>
+        </is>
+      </c>
+      <c r="D8" s="5" t="n"/>
+    </row>
+    <row r="9" ht="50" customHeight="1">
+      <c r="B9" s="18" t="inlineStr">
+        <is>
+          <t>5. Do not infer unsupported clinical relationships.</t>
+        </is>
+      </c>
+      <c r="C9" s="19" t="inlineStr">
+        <is>
+          <t>Use only information expressed or clearly established in the narrative. Do not infer causality, chronology, indication, manifestation, or treatment role solely from medical knowledge.</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="n"/>
+    </row>
+    <row r="10" ht="50" customHeight="1">
+      <c r="B10" s="20" t="inlineStr">
+        <is>
+          <t>6. Do not annotate the same text span with multiple categories.</t>
+        </is>
+      </c>
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>Choose the category that best represents the role of that span in its local narrative context.</t>
+        </is>
+      </c>
+      <c r="D10" s="5" t="n"/>
+    </row>
+    <row r="11" ht="50" customHeight="1">
+      <c r="B11" s="18" t="inlineStr">
+        <is>
+          <t>7. Do not create overlapping or nested annotations.</t>
+        </is>
+      </c>
+      <c r="C11" s="19" t="inlineStr"/>
+      <c r="D11" s="5" t="n"/>
+    </row>
+    <row r="12" ht="50" customHeight="1">
+      <c r="B12" s="20" t="inlineStr">
+        <is>
+          <t>8. Drug-role precedence must be contextual.</t>
+        </is>
+      </c>
+      <c r="C12" s="21" t="inlineStr">
+        <is>
+          <t>For each drug mention, determine its role in that specific context:
+- sDrug = suspected or implicated in causing/contributing to an AE.
+- cDrug = concurrent/background medication.
+- Treatment = explicitly administered to treat a disease, AE, complication, or symptom.
+- oDrug = drug mentioned without sufficient evidence for the above roles.</t>
+        </is>
+      </c>
+      <c r="D12" s="5" t="n"/>
+    </row>
+    <row r="13" ht="50" customHeight="1">
+      <c r="B13" s="18" t="inlineStr">
+        <is>
+          <t>9. AE versus mAE must be based on an explicit relationship.</t>
+        </is>
+      </c>
+      <c r="C13" s="19" t="inlineStr">
+        <is>
+          <t>- AE = the adverse health event/condition/symptom itself.
+- mAE = a manifestation, complication, consequence, or sequela explicitly linked to another AE.
+If that relationship is not established in the narrative, do not infer mAE.</t>
+        </is>
+      </c>
+      <c r="D13" s="5" t="n"/>
+    </row>
+    <row r="14" ht="50" customHeight="1">
+      <c r="B14" s="20" t="inlineStr">
+        <is>
+          <t>10. AE versus MHx is determined by temporal/contextual role.</t>
+        </is>
+      </c>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>A condition explicitly described as pre-existing, chronic, baseline, or historical should be MHx rather than AE in that occurrence.</t>
+        </is>
+      </c>
+      <c r="D14" s="5" t="n"/>
+    </row>
+    <row r="15" ht="50" customHeight="1">
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>11. IND is the reason for treatment, not the treatment itself.</t>
+        </is>
+      </c>
+      <c r="C15" s="19" t="inlineStr">
+        <is>
+          <t>Example:
+"prednisone for rash"
+- "prednisone" -&gt; Treatment when explicitly being used therapeutically.
+- "rash" -&gt; IND when explicitly stated as the reason for prednisone.</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="n"/>
+    </row>
+    <row r="16" ht="50" customHeight="1">
+      <c r="B16" s="20" t="inlineStr">
+        <is>
+          <t>12. Dx versus Lab:</t>
+        </is>
+      </c>
+      <c r="C16" s="21" t="inlineStr">
+        <is>
+          <t>- Dx = diagnostic procedure.
+- Lab = laboratory test, measurement, or laboratory finding/result.</t>
+        </is>
+      </c>
+      <c r="D16" s="5" t="n"/>
+    </row>
+    <row r="17" ht="50" customHeight="1">
+      <c r="B17" s="18" t="inlineStr">
+        <is>
+          <t>13. Status describes clinical course or outcome.</t>
+        </is>
+      </c>
+      <c r="C17" s="19" t="inlineStr">
+        <is>
+          <t>Do not label the underlying disease or AE as Status merely because its outcome is discussed.</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="n"/>
+    </row>
+    <row r="18" ht="50" customHeight="1">
+      <c r="B18" s="20" t="inlineStr">
+        <is>
+          <t>14. Repeated mentions may be annotated separately.</t>
+        </is>
+      </c>
+      <c r="C18" s="21" t="inlineStr">
+        <is>
+          <t>If the same clinical concept appears multiple times in the narrative, annotate each explicit occurrence according to its local context.</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="n"/>
+    </row>
+    <row r="19" ht="50" customHeight="1">
+      <c r="B19" s="18" t="inlineStr">
+        <is>
+          <t>15. Annotate only the 17 categories defined above.</t>
+        </is>
+      </c>
+      <c r="C19" s="19" t="inlineStr">
+        <is>
+          <t>Do not invent or add additional categories.</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="17">
+    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="C6:D6"/>
+    <mergeCell ref="C7:D7"/>
+    <mergeCell ref="C10:D10"/>
+    <mergeCell ref="C8:D8"/>
+    <mergeCell ref="C15:D15"/>
+    <mergeCell ref="C16:D16"/>
+    <mergeCell ref="C11:D11"/>
+    <mergeCell ref="C5:D5"/>
+    <mergeCell ref="C19:D19"/>
+    <mergeCell ref="C14:D14"/>
+    <mergeCell ref="C13:D13"/>
+    <mergeCell ref="C9:D9"/>
+    <mergeCell ref="C17:D17"/>
+    <mergeCell ref="C18:D18"/>
     <mergeCell ref="B2:D2"/>
+    <mergeCell ref="C4:D4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>